<commit_message>
Add project dashboard and validation UI
</commit_message>
<xml_diff>
--- a/docs/Template.xlsx
+++ b/docs/Template.xlsx
@@ -8,16 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alcoberr\Documents\Work in progress code\prototype_pictures\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69E1199B-FE8E-4FAC-BD3F-1421076F38C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C95CAFE5-B08D-4DFC-AC4B-EE71E1767111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19120" yWindow="10690" windowWidth="23260" windowHeight="14860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11630" yWindow="10690" windowWidth="23260" windowHeight="14860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Appendix B - Pictures" sheetId="8" r:id="rId1"/>
+    <sheet name="Page 1" sheetId="10" r:id="rId1"/>
+    <sheet name="Page 2" sheetId="8" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Appendix B - Pictures'!$D$1:$AQ$92</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Appendix B - Pictures'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Page 1'!$D$1:$AQ$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Page 2'!$D$1:$AQ$46</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Page 1'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Page 2'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="10">
   <si>
     <t>WORK ORDER:</t>
   </si>
@@ -48,16 +51,22 @@
     <t>VISUAL INSPECTION AND SUPPORTING PICTURE(S)</t>
   </si>
   <si>
-    <t xml:space="preserve">FIGURE 01: Tank Construction </t>
+    <t>IMG_TOP_1</t>
   </si>
   <si>
-    <t>FIGURE 02: BAY-O-NET FUSES</t>
+    <t>IMG_TOP_2</t>
   </si>
   <si>
-    <t xml:space="preserve">FIGURE 04: </t>
+    <t>IMG_BOTTOM_1</t>
   </si>
   <si>
-    <t xml:space="preserve">FIGURE 03: </t>
+    <t>IMG_BOTTOM_2</t>
+  </si>
+  <si>
+    <t>FIGURE_TOP</t>
+  </si>
+  <si>
+    <t>FIGURE_BOTTOM</t>
   </si>
 </sst>
 </file>
@@ -240,7 +249,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -249,6 +258,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -260,6 +272,18 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -267,6 +291,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -281,27 +314,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -346,10 +358,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="25798" name="Picture 4" descr="logo948_grey+30_12">
+        <xdr:cNvPr id="2" name="Picture 4" descr="logo948_grey+30_12">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9A3A86B-5947-4851-812C-7E823B83DED9}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9E4B90C-92D5-43DD-B777-67740F478AAC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -372,8 +384,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="15520149" y="66855"/>
-          <a:ext cx="1441648" cy="1468351"/>
+          <a:off x="40614602" y="66855"/>
+          <a:ext cx="1364327" cy="1470032"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -420,10 +432,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="25803" name="Picture 493">
+        <xdr:cNvPr id="3" name="Picture 493">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7E254A1C-5DDE-409A-BE6E-72EBABFFF5CD}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E08E0A9B-4AE3-4484-90E7-4E46147D1C51}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -446,8 +458,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="65919" y="56030"/>
-          <a:ext cx="1973551" cy="1514299"/>
+          <a:off x="26088219" y="56030"/>
+          <a:ext cx="1870457" cy="1515980"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -768,6 +780,540 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D76EE82-9938-4754-8B62-6CDD61F8DBAE}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="D1:BE157"/>
+  <sheetFormatPr defaultColWidth="6.7109375" defaultRowHeight="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="255.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="128.140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="6.7109375" style="2"/>
+    <col min="4" max="43" width="6" style="2" customWidth="1"/>
+    <col min="44" max="16384" width="6.7109375" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D1" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13"/>
+      <c r="S1" s="13"/>
+      <c r="T1" s="13"/>
+      <c r="U1" s="13"/>
+      <c r="V1" s="13"/>
+      <c r="W1" s="13"/>
+      <c r="X1" s="13"/>
+      <c r="Y1" s="13"/>
+      <c r="Z1" s="13"/>
+      <c r="AA1" s="13"/>
+      <c r="AB1" s="13"/>
+      <c r="AC1" s="13"/>
+      <c r="AD1" s="13"/>
+      <c r="AE1" s="13"/>
+      <c r="AF1" s="13"/>
+      <c r="AG1" s="13"/>
+      <c r="AH1" s="13"/>
+      <c r="AI1" s="13"/>
+      <c r="AJ1" s="13"/>
+      <c r="AK1" s="13"/>
+      <c r="AL1" s="13"/>
+      <c r="AM1" s="13"/>
+      <c r="AN1" s="13"/>
+      <c r="AO1" s="13"/>
+      <c r="AP1" s="13"/>
+      <c r="AQ1" s="14"/>
+    </row>
+    <row r="2" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D2" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16"/>
+      <c r="Q2" s="16"/>
+      <c r="R2" s="16"/>
+      <c r="S2" s="16"/>
+      <c r="T2" s="16"/>
+      <c r="U2" s="16"/>
+      <c r="V2" s="16"/>
+      <c r="W2" s="16"/>
+      <c r="X2" s="16"/>
+      <c r="Y2" s="16"/>
+      <c r="Z2" s="16"/>
+      <c r="AA2" s="16"/>
+      <c r="AB2" s="16"/>
+      <c r="AC2" s="16"/>
+      <c r="AD2" s="16"/>
+      <c r="AE2" s="16"/>
+      <c r="AF2" s="16"/>
+      <c r="AG2" s="16"/>
+      <c r="AH2" s="16"/>
+      <c r="AI2" s="16"/>
+      <c r="AJ2" s="16"/>
+      <c r="AK2" s="16"/>
+      <c r="AL2" s="16"/>
+      <c r="AM2" s="16"/>
+      <c r="AN2" s="16"/>
+      <c r="AO2" s="16"/>
+      <c r="AP2" s="16"/>
+      <c r="AQ2" s="17"/>
+    </row>
+    <row r="3" spans="4:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D3" s="15"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="20"/>
+      <c r="Q3" s="21"/>
+      <c r="R3" s="21"/>
+      <c r="S3" s="21"/>
+      <c r="T3" s="21"/>
+      <c r="U3" s="21"/>
+      <c r="V3" s="21"/>
+      <c r="W3" s="21"/>
+      <c r="X3" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y3" s="18"/>
+      <c r="Z3" s="18"/>
+      <c r="AA3" s="18"/>
+      <c r="AB3" s="18"/>
+      <c r="AC3" s="18"/>
+      <c r="AD3" s="20"/>
+      <c r="AE3" s="22"/>
+      <c r="AF3" s="22"/>
+      <c r="AG3" s="22"/>
+      <c r="AH3" s="22"/>
+      <c r="AI3" s="22"/>
+      <c r="AJ3" s="22"/>
+      <c r="AK3" s="22"/>
+      <c r="AL3" s="23"/>
+      <c r="AM3" s="23"/>
+      <c r="AN3" s="23"/>
+      <c r="AO3" s="23"/>
+      <c r="AP3" s="23"/>
+      <c r="AQ3" s="24"/>
+    </row>
+    <row r="4" spans="4:43" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D4" s="8"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="9"/>
+      <c r="P4" s="9"/>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9"/>
+      <c r="S4" s="9"/>
+      <c r="T4" s="9"/>
+      <c r="U4" s="9"/>
+      <c r="V4" s="9"/>
+      <c r="W4" s="9"/>
+      <c r="X4" s="9"/>
+      <c r="Y4" s="9"/>
+      <c r="Z4" s="9"/>
+      <c r="AA4" s="9"/>
+      <c r="AB4" s="9"/>
+      <c r="AC4" s="9"/>
+      <c r="AD4" s="9"/>
+      <c r="AE4" s="9"/>
+      <c r="AF4" s="9"/>
+      <c r="AG4" s="9"/>
+      <c r="AH4" s="9"/>
+      <c r="AI4" s="9"/>
+      <c r="AJ4" s="9"/>
+      <c r="AK4" s="9"/>
+      <c r="AL4" s="9"/>
+      <c r="AM4" s="9"/>
+      <c r="AN4" s="9"/>
+      <c r="AO4" s="9"/>
+      <c r="AP4" s="9"/>
+      <c r="AQ4" s="10"/>
+    </row>
+    <row r="5" spans="4:43" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
+      <c r="N5" s="11"/>
+      <c r="O5" s="11"/>
+      <c r="P5" s="11"/>
+      <c r="Q5" s="11"/>
+      <c r="R5" s="11"/>
+      <c r="S5" s="11"/>
+      <c r="T5" s="11"/>
+      <c r="U5" s="11"/>
+      <c r="V5" s="11"/>
+      <c r="W5" s="11"/>
+      <c r="X5" s="11"/>
+      <c r="Y5" s="11"/>
+      <c r="Z5" s="11"/>
+      <c r="AA5" s="11"/>
+      <c r="AB5" s="11"/>
+      <c r="AC5" s="11"/>
+      <c r="AD5" s="11"/>
+      <c r="AE5" s="11"/>
+      <c r="AF5" s="11"/>
+      <c r="AG5" s="11"/>
+      <c r="AH5" s="11"/>
+      <c r="AI5" s="11"/>
+      <c r="AJ5" s="11"/>
+      <c r="AK5" s="11"/>
+      <c r="AL5" s="11"/>
+      <c r="AM5" s="11"/>
+      <c r="AN5" s="11"/>
+      <c r="AO5" s="11"/>
+      <c r="AP5" s="11"/>
+      <c r="AQ5" s="11"/>
+    </row>
+    <row r="6" spans="4:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="6"/>
+      <c r="T6" s="6"/>
+      <c r="U6" s="6"/>
+      <c r="V6" s="6"/>
+      <c r="W6" s="6"/>
+      <c r="X6" s="6"/>
+      <c r="Y6" s="6"/>
+      <c r="Z6" s="6"/>
+      <c r="AA6" s="6"/>
+      <c r="AB6" s="6"/>
+      <c r="AC6" s="6"/>
+      <c r="AD6" s="6"/>
+      <c r="AE6" s="6"/>
+      <c r="AF6" s="6"/>
+      <c r="AG6" s="6"/>
+      <c r="AH6" s="6"/>
+      <c r="AI6" s="6"/>
+      <c r="AJ6" s="6"/>
+      <c r="AK6" s="6"/>
+      <c r="AL6" s="6"/>
+      <c r="AM6" s="6"/>
+      <c r="AN6" s="6"/>
+      <c r="AO6" s="6"/>
+      <c r="AP6" s="6"/>
+      <c r="AQ6" s="7"/>
+    </row>
+    <row r="7" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D7"/>
+      <c r="AQ7" s="1"/>
+    </row>
+    <row r="8" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D8" s="3"/>
+      <c r="AQ8" s="1"/>
+    </row>
+    <row r="9" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D9" s="3"/>
+      <c r="AQ9" s="1"/>
+    </row>
+    <row r="10" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D10" s="3"/>
+      <c r="G10" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AA10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="AQ10" s="1"/>
+    </row>
+    <row r="11" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D11" s="3"/>
+      <c r="AQ11" s="1"/>
+    </row>
+    <row r="12" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D12" s="3"/>
+      <c r="AQ12" s="1"/>
+    </row>
+    <row r="13" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D13" s="3"/>
+      <c r="AQ13" s="1"/>
+    </row>
+    <row r="14" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D14" s="3"/>
+      <c r="AQ14" s="1"/>
+    </row>
+    <row r="15" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D15" s="3"/>
+      <c r="AQ15" s="1"/>
+    </row>
+    <row r="16" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D16" s="3"/>
+      <c r="AQ16" s="1"/>
+    </row>
+    <row r="17" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D17" s="3"/>
+      <c r="AQ17" s="1"/>
+    </row>
+    <row r="18" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D18" s="3"/>
+      <c r="AQ18" s="1"/>
+    </row>
+    <row r="19" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D19" s="3"/>
+      <c r="AQ19" s="1"/>
+    </row>
+    <row r="20" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D20" s="3"/>
+      <c r="AQ20" s="1"/>
+    </row>
+    <row r="21" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D21" s="3"/>
+      <c r="AQ21" s="1"/>
+    </row>
+    <row r="22" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D22" s="3"/>
+      <c r="AQ22" s="1"/>
+    </row>
+    <row r="23" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D23" s="3"/>
+      <c r="AQ23" s="1"/>
+    </row>
+    <row r="24" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D24" s="3"/>
+      <c r="AQ24" s="1"/>
+    </row>
+    <row r="25" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D25" s="3"/>
+      <c r="AQ25" s="1"/>
+    </row>
+    <row r="26" spans="4:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D26" s="3"/>
+      <c r="AQ26" s="1"/>
+    </row>
+    <row r="27" spans="4:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D27" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="6"/>
+      <c r="K27" s="6"/>
+      <c r="L27" s="6"/>
+      <c r="M27" s="6"/>
+      <c r="N27" s="6"/>
+      <c r="O27" s="6"/>
+      <c r="P27" s="6"/>
+      <c r="Q27" s="6"/>
+      <c r="R27" s="6"/>
+      <c r="S27" s="6"/>
+      <c r="T27" s="6"/>
+      <c r="U27" s="6"/>
+      <c r="V27" s="6"/>
+      <c r="W27" s="6"/>
+      <c r="X27" s="6"/>
+      <c r="Y27" s="6"/>
+      <c r="Z27" s="6"/>
+      <c r="AA27" s="6"/>
+      <c r="AB27" s="6"/>
+      <c r="AC27" s="6"/>
+      <c r="AD27" s="6"/>
+      <c r="AE27" s="6"/>
+      <c r="AF27" s="6"/>
+      <c r="AG27" s="6"/>
+      <c r="AH27" s="6"/>
+      <c r="AI27" s="6"/>
+      <c r="AJ27" s="6"/>
+      <c r="AK27" s="6"/>
+      <c r="AL27" s="6"/>
+      <c r="AM27" s="6"/>
+      <c r="AN27" s="6"/>
+      <c r="AO27" s="6"/>
+      <c r="AP27" s="6"/>
+      <c r="AQ27" s="7"/>
+    </row>
+    <row r="28" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D28" s="3"/>
+      <c r="AQ28" s="1"/>
+    </row>
+    <row r="29" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D29" s="3"/>
+      <c r="AQ29" s="1"/>
+    </row>
+    <row r="30" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D30" s="3"/>
+      <c r="AQ30" s="1"/>
+    </row>
+    <row r="31" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D31" s="3"/>
+      <c r="G31" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="Z31" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="AK31"/>
+      <c r="AQ31" s="1"/>
+    </row>
+    <row r="32" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D32" s="3"/>
+      <c r="AQ32" s="1"/>
+    </row>
+    <row r="33" spans="4:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D33" s="3"/>
+      <c r="AQ33" s="1"/>
+    </row>
+    <row r="34" spans="4:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D34" s="3"/>
+      <c r="AQ34" s="1"/>
+    </row>
+    <row r="35" spans="4:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D35" s="3"/>
+      <c r="AQ35" s="1"/>
+      <c r="AZ35"/>
+    </row>
+    <row r="36" spans="4:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D36" s="3"/>
+      <c r="AQ36" s="1"/>
+    </row>
+    <row r="37" spans="4:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D37" s="3"/>
+      <c r="AQ37" s="1"/>
+    </row>
+    <row r="38" spans="4:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D38" s="3"/>
+      <c r="AQ38" s="1"/>
+    </row>
+    <row r="39" spans="4:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D39" s="3"/>
+      <c r="AQ39" s="1"/>
+    </row>
+    <row r="40" spans="4:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D40" s="3"/>
+      <c r="AQ40" s="1"/>
+    </row>
+    <row r="41" spans="4:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D41" s="3"/>
+      <c r="AQ41" s="1"/>
+    </row>
+    <row r="42" spans="4:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D42" s="3"/>
+      <c r="AQ42" s="1"/>
+    </row>
+    <row r="43" spans="4:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D43" s="3"/>
+      <c r="AQ43" s="1"/>
+    </row>
+    <row r="44" spans="4:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D44" s="3"/>
+      <c r="AQ44" s="1"/>
+    </row>
+    <row r="45" spans="4:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D45" s="3"/>
+      <c r="AQ45" s="1"/>
+    </row>
+    <row r="46" spans="4:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D46" s="3"/>
+      <c r="AQ46" s="1"/>
+    </row>
+    <row r="47" spans="4:52" ht="26.1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="4:52" ht="36.6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="52:52" ht="23.25" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="52:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AZ77"/>
+    </row>
+    <row r="91" spans="53:53" ht="23.25" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="53:53" ht="23.25" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="53:53" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BA93"/>
+    </row>
+    <row r="114" spans="57:57" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="121" spans="57:57" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BE121"/>
+    </row>
+    <row r="135" ht="23.25" x14ac:dyDescent="0.25"/>
+    <row r="136" ht="23.25" x14ac:dyDescent="0.25"/>
+    <row r="157" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="D4:AQ4"/>
+    <mergeCell ref="D5:AQ5"/>
+    <mergeCell ref="D6:AQ6"/>
+    <mergeCell ref="D27:AQ27"/>
+    <mergeCell ref="D1:AQ1"/>
+    <mergeCell ref="D2:AQ2"/>
+    <mergeCell ref="D3:J3"/>
+    <mergeCell ref="K3:O3"/>
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:AC3"/>
+    <mergeCell ref="AD3:AK3"/>
+    <mergeCell ref="AL3:AQ3"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>
+  <pageSetup scale="42" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <headerFooter scaleWithDoc="0" alignWithMargins="0">
+    <oddFooter>&amp;L&amp;"Arial,Bold"&amp;12Appendix B &amp;"Arial,Regular"- Page &amp;"Arial,Bold"&amp;P &amp;"Arial,Regular"of&amp;"Arial,Bold" &amp;N&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;22&amp;K0073CF INTERNAL</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
@@ -782,279 +1328,387 @@
     <col min="44" max="16384" width="6.7109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D1" s="7" t="s">
-        <v>2</v>
+    <row r="1" spans="4:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D1" s="5" t="s">
+        <v>8</v>
       </c>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="8"/>
-      <c r="R1" s="8"/>
-      <c r="S1" s="8"/>
-      <c r="T1" s="8"/>
-      <c r="U1" s="8"/>
-      <c r="V1" s="8"/>
-      <c r="W1" s="8"/>
-      <c r="X1" s="8"/>
-      <c r="Y1" s="8"/>
-      <c r="Z1" s="8"/>
-      <c r="AA1" s="8"/>
-      <c r="AB1" s="8"/>
-      <c r="AC1" s="8"/>
-      <c r="AD1" s="8"/>
-      <c r="AE1" s="8"/>
-      <c r="AF1" s="8"/>
-      <c r="AG1" s="8"/>
-      <c r="AH1" s="8"/>
-      <c r="AI1" s="8"/>
-      <c r="AJ1" s="8"/>
-      <c r="AK1" s="8"/>
-      <c r="AL1" s="8"/>
-      <c r="AM1" s="8"/>
-      <c r="AN1" s="8"/>
-      <c r="AO1" s="8"/>
-      <c r="AP1" s="8"/>
-      <c r="AQ1" s="9"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6"/>
+      <c r="T1" s="6"/>
+      <c r="U1" s="6"/>
+      <c r="V1" s="6"/>
+      <c r="W1" s="6"/>
+      <c r="X1" s="6"/>
+      <c r="Y1" s="6"/>
+      <c r="Z1" s="6"/>
+      <c r="AA1" s="6"/>
+      <c r="AB1" s="6"/>
+      <c r="AC1" s="6"/>
+      <c r="AD1" s="6"/>
+      <c r="AE1" s="6"/>
+      <c r="AF1" s="6"/>
+      <c r="AG1" s="6"/>
+      <c r="AH1" s="6"/>
+      <c r="AI1" s="6"/>
+      <c r="AJ1" s="6"/>
+      <c r="AK1" s="6"/>
+      <c r="AL1" s="6"/>
+      <c r="AM1" s="6"/>
+      <c r="AN1" s="6"/>
+      <c r="AO1" s="6"/>
+      <c r="AP1" s="6"/>
+      <c r="AQ1" s="7"/>
     </row>
     <row r="2" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D2" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-      <c r="N2" s="20"/>
-      <c r="O2" s="20"/>
-      <c r="P2" s="20"/>
-      <c r="Q2" s="20"/>
-      <c r="R2" s="20"/>
-      <c r="S2" s="20"/>
-      <c r="T2" s="20"/>
-      <c r="U2" s="20"/>
-      <c r="V2" s="20"/>
-      <c r="W2" s="20"/>
-      <c r="X2" s="20"/>
-      <c r="Y2" s="20"/>
-      <c r="Z2" s="20"/>
-      <c r="AA2" s="20"/>
-      <c r="AB2" s="20"/>
-      <c r="AC2" s="20"/>
-      <c r="AD2" s="20"/>
-      <c r="AE2" s="20"/>
-      <c r="AF2" s="20"/>
-      <c r="AG2" s="20"/>
-      <c r="AH2" s="20"/>
-      <c r="AI2" s="20"/>
-      <c r="AJ2" s="20"/>
-      <c r="AK2" s="20"/>
-      <c r="AL2" s="20"/>
-      <c r="AM2" s="20"/>
-      <c r="AN2" s="20"/>
-      <c r="AO2" s="20"/>
-      <c r="AP2" s="20"/>
-      <c r="AQ2" s="21"/>
-    </row>
-    <row r="3" spans="4:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D3" s="19"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
-      <c r="K3" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="13"/>
-      <c r="R3" s="13"/>
-      <c r="S3" s="13"/>
-      <c r="T3" s="13"/>
-      <c r="U3" s="13"/>
-      <c r="V3" s="13"/>
-      <c r="W3" s="13"/>
-      <c r="X3" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="Y3" s="10"/>
-      <c r="Z3" s="10"/>
-      <c r="AA3" s="10"/>
-      <c r="AB3" s="10"/>
-      <c r="AC3" s="10"/>
-      <c r="AD3" s="12"/>
-      <c r="AE3" s="14"/>
-      <c r="AF3" s="14"/>
-      <c r="AG3" s="14"/>
-      <c r="AH3" s="14"/>
-      <c r="AI3" s="14"/>
-      <c r="AJ3" s="14"/>
-      <c r="AK3" s="14"/>
-      <c r="AL3" s="22"/>
-      <c r="AM3" s="22"/>
-      <c r="AN3" s="22"/>
-      <c r="AO3" s="22"/>
-      <c r="AP3" s="22"/>
-      <c r="AQ3" s="23"/>
-    </row>
-    <row r="4" spans="4:43" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D4" s="16"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="17"/>
-      <c r="O4" s="17"/>
-      <c r="P4" s="17"/>
-      <c r="Q4" s="17"/>
-      <c r="R4" s="17"/>
-      <c r="S4" s="17"/>
-      <c r="T4" s="17"/>
-      <c r="U4" s="17"/>
-      <c r="V4" s="17"/>
-      <c r="W4" s="17"/>
-      <c r="X4" s="17"/>
-      <c r="Y4" s="17"/>
-      <c r="Z4" s="17"/>
-      <c r="AA4" s="17"/>
-      <c r="AB4" s="17"/>
-      <c r="AC4" s="17"/>
-      <c r="AD4" s="17"/>
-      <c r="AE4" s="17"/>
-      <c r="AF4" s="17"/>
-      <c r="AG4" s="17"/>
-      <c r="AH4" s="17"/>
-      <c r="AI4" s="17"/>
-      <c r="AJ4" s="17"/>
-      <c r="AK4" s="17"/>
-      <c r="AL4" s="17"/>
-      <c r="AM4" s="17"/>
-      <c r="AN4" s="17"/>
-      <c r="AO4" s="17"/>
-      <c r="AP4" s="17"/>
-      <c r="AQ4" s="18"/>
-    </row>
-    <row r="5" spans="4:43" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
-      <c r="R5" s="15"/>
-      <c r="S5" s="15"/>
-      <c r="T5" s="15"/>
-      <c r="U5" s="15"/>
-      <c r="V5" s="15"/>
-      <c r="W5" s="15"/>
-      <c r="X5" s="15"/>
-      <c r="Y5" s="15"/>
-      <c r="Z5" s="15"/>
-      <c r="AA5" s="15"/>
-      <c r="AB5" s="15"/>
-      <c r="AC5" s="15"/>
-      <c r="AD5" s="15"/>
-      <c r="AE5" s="15"/>
-      <c r="AF5" s="15"/>
-      <c r="AG5" s="15"/>
-      <c r="AH5" s="15"/>
-      <c r="AI5" s="15"/>
-      <c r="AJ5" s="15"/>
-      <c r="AK5" s="15"/>
-      <c r="AL5" s="15"/>
-      <c r="AM5" s="15"/>
-      <c r="AN5" s="15"/>
-      <c r="AO5" s="15"/>
-      <c r="AP5" s="15"/>
-      <c r="AQ5" s="15"/>
-    </row>
-    <row r="6" spans="4:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D6" s="4" t="s">
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
+      <c r="V2" s="4"/>
+      <c r="W2" s="4"/>
+      <c r="X2" s="4"/>
+      <c r="Y2" s="4"/>
+      <c r="Z2" s="4"/>
+      <c r="AA2" s="4"/>
+      <c r="AB2" s="4"/>
+      <c r="AC2" s="4"/>
+      <c r="AD2" s="4"/>
+      <c r="AE2" s="4"/>
+      <c r="AF2" s="4"/>
+      <c r="AG2" s="4"/>
+      <c r="AH2" s="4"/>
+      <c r="AI2" s="4"/>
+      <c r="AJ2" s="4"/>
+      <c r="AK2" s="4"/>
+      <c r="AL2" s="4"/>
+      <c r="AM2" s="4"/>
+      <c r="AN2" s="4"/>
+      <c r="AO2" s="4"/>
+      <c r="AP2" s="4"/>
+      <c r="AQ2" s="4"/>
+    </row>
+    <row r="3" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4"/>
+      <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+      <c r="V3" s="4"/>
+      <c r="W3" s="4"/>
+      <c r="X3" s="4"/>
+      <c r="Y3" s="4"/>
+      <c r="Z3" s="4"/>
+      <c r="AA3" s="4"/>
+      <c r="AB3" s="4"/>
+      <c r="AC3" s="4"/>
+      <c r="AD3" s="4"/>
+      <c r="AE3" s="4"/>
+      <c r="AF3" s="4"/>
+      <c r="AG3" s="4"/>
+      <c r="AH3" s="4"/>
+      <c r="AI3" s="4"/>
+      <c r="AJ3" s="4"/>
+      <c r="AK3" s="4"/>
+      <c r="AL3" s="4"/>
+      <c r="AM3" s="4"/>
+      <c r="AN3" s="4"/>
+      <c r="AO3" s="4"/>
+      <c r="AP3" s="4"/>
+      <c r="AQ3" s="4"/>
+    </row>
+    <row r="4" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
+      <c r="W4" s="4"/>
+      <c r="X4" s="4"/>
+      <c r="Y4" s="4"/>
+      <c r="Z4" s="4"/>
+      <c r="AA4" s="4"/>
+      <c r="AB4" s="4"/>
+      <c r="AC4" s="4"/>
+      <c r="AD4" s="4"/>
+      <c r="AE4" s="4"/>
+      <c r="AF4" s="4"/>
+      <c r="AG4" s="4"/>
+      <c r="AH4" s="4"/>
+      <c r="AI4" s="4"/>
+      <c r="AJ4" s="4"/>
+      <c r="AK4" s="4"/>
+      <c r="AL4" s="4"/>
+      <c r="AM4" s="4"/>
+      <c r="AN4" s="4"/>
+      <c r="AO4" s="4"/>
+      <c r="AP4" s="4"/>
+      <c r="AQ4" s="4"/>
+    </row>
+    <row r="5" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
+      <c r="V5" s="4"/>
+      <c r="W5" s="4"/>
+      <c r="X5" s="4"/>
+      <c r="Y5" s="4"/>
+      <c r="Z5" s="4"/>
+      <c r="AA5" s="4"/>
+      <c r="AB5" s="4"/>
+      <c r="AC5" s="4"/>
+      <c r="AD5" s="4"/>
+      <c r="AE5" s="4"/>
+      <c r="AF5" s="4"/>
+      <c r="AG5" s="4"/>
+      <c r="AH5" s="4"/>
+      <c r="AI5" s="4"/>
+      <c r="AJ5" s="4"/>
+      <c r="AK5" s="4"/>
+      <c r="AL5" s="4"/>
+      <c r="AM5" s="4"/>
+      <c r="AN5" s="4"/>
+      <c r="AO5" s="4"/>
+      <c r="AP5" s="4"/>
+      <c r="AQ5" s="4"/>
+    </row>
+    <row r="6" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="5"/>
-      <c r="R6" s="5"/>
-      <c r="S6" s="5"/>
-      <c r="T6" s="5"/>
-      <c r="U6" s="5"/>
-      <c r="V6" s="5"/>
-      <c r="W6" s="5"/>
-      <c r="X6" s="5"/>
-      <c r="Y6" s="5"/>
-      <c r="Z6" s="5"/>
-      <c r="AA6" s="5"/>
-      <c r="AB6" s="5"/>
-      <c r="AC6" s="5"/>
-      <c r="AD6" s="5"/>
-      <c r="AE6" s="5"/>
-      <c r="AF6" s="5"/>
-      <c r="AG6" s="5"/>
-      <c r="AH6" s="5"/>
-      <c r="AI6" s="5"/>
-      <c r="AJ6" s="5"/>
-      <c r="AK6" s="5"/>
-      <c r="AL6" s="5"/>
-      <c r="AM6" s="5"/>
-      <c r="AN6" s="5"/>
-      <c r="AO6" s="5"/>
-      <c r="AP6" s="5"/>
-      <c r="AQ6" s="6"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="4"/>
+      <c r="T6" s="4"/>
+      <c r="U6" s="4"/>
+      <c r="V6" s="4"/>
+      <c r="W6" s="4"/>
+      <c r="X6" s="4"/>
+      <c r="Y6" s="4"/>
+      <c r="Z6" s="4"/>
+      <c r="AA6" s="4"/>
+      <c r="AB6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="AC6" s="4"/>
+      <c r="AE6" s="4"/>
+      <c r="AF6" s="4"/>
+      <c r="AG6" s="4"/>
+      <c r="AH6" s="4"/>
+      <c r="AI6" s="4"/>
+      <c r="AJ6" s="4"/>
+      <c r="AK6" s="4"/>
+      <c r="AL6" s="4"/>
+      <c r="AM6" s="4"/>
+      <c r="AN6" s="4"/>
+      <c r="AO6" s="4"/>
+      <c r="AP6" s="4"/>
+      <c r="AQ6" s="4"/>
     </row>
     <row r="7" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D7"/>
-      <c r="AQ7" s="1"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
+      <c r="R7" s="4"/>
+      <c r="S7" s="4"/>
+      <c r="T7" s="4"/>
+      <c r="U7" s="4"/>
+      <c r="V7" s="4"/>
+      <c r="W7" s="4"/>
+      <c r="X7" s="4"/>
+      <c r="Y7" s="4"/>
+      <c r="Z7" s="4"/>
+      <c r="AA7" s="4"/>
+      <c r="AB7" s="4"/>
+      <c r="AC7" s="4"/>
+      <c r="AD7" s="4"/>
+      <c r="AE7" s="4"/>
+      <c r="AF7" s="4"/>
+      <c r="AG7" s="4"/>
+      <c r="AH7" s="4"/>
+      <c r="AI7" s="4"/>
+      <c r="AJ7" s="4"/>
+      <c r="AK7" s="4"/>
+      <c r="AL7" s="4"/>
+      <c r="AM7" s="4"/>
+      <c r="AN7" s="4"/>
+      <c r="AO7" s="4"/>
+      <c r="AP7" s="4"/>
+      <c r="AQ7" s="4"/>
     </row>
     <row r="8" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D8" s="3"/>
-      <c r="AQ8" s="1"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
+      <c r="S8" s="4"/>
+      <c r="T8" s="4"/>
+      <c r="U8" s="4"/>
+      <c r="V8" s="4"/>
+      <c r="W8" s="4"/>
+      <c r="X8" s="4"/>
+      <c r="Y8" s="4"/>
+      <c r="Z8" s="4"/>
+      <c r="AA8" s="4"/>
+      <c r="AB8" s="4"/>
+      <c r="AC8" s="4"/>
+      <c r="AD8" s="4"/>
+      <c r="AE8" s="4"/>
+      <c r="AF8" s="4"/>
+      <c r="AG8" s="4"/>
+      <c r="AH8" s="4"/>
+      <c r="AI8" s="4"/>
+      <c r="AJ8" s="4"/>
+      <c r="AK8" s="4"/>
+      <c r="AL8" s="4"/>
+      <c r="AM8" s="4"/>
+      <c r="AN8" s="4"/>
+      <c r="AO8" s="4"/>
+      <c r="AP8" s="4"/>
+      <c r="AQ8" s="4"/>
     </row>
     <row r="9" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D9" s="3"/>
-      <c r="AQ9" s="1"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
+      <c r="R9" s="4"/>
+      <c r="S9" s="4"/>
+      <c r="T9" s="4"/>
+      <c r="U9" s="4"/>
+      <c r="V9" s="4"/>
+      <c r="W9" s="4"/>
+      <c r="X9" s="4"/>
+      <c r="Y9" s="4"/>
+      <c r="Z9" s="4"/>
+      <c r="AA9" s="4"/>
+      <c r="AB9" s="4"/>
+      <c r="AC9" s="4"/>
+      <c r="AD9" s="4"/>
+      <c r="AE9" s="4"/>
+      <c r="AF9" s="4"/>
+      <c r="AG9" s="4"/>
+      <c r="AH9" s="4"/>
+      <c r="AI9" s="4"/>
+      <c r="AJ9" s="4"/>
+      <c r="AK9" s="4"/>
+      <c r="AL9" s="4"/>
+      <c r="AM9" s="4"/>
+      <c r="AN9" s="4"/>
+      <c r="AO9" s="4"/>
+      <c r="AP9" s="4"/>
+      <c r="AQ9" s="4"/>
     </row>
     <row r="10" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D10" s="3"/>
@@ -1104,13 +1758,53 @@
       <c r="D21" s="3"/>
       <c r="AQ21" s="1"/>
     </row>
-    <row r="22" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="4:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D22" s="3"/>
       <c r="AQ22" s="1"/>
     </row>
-    <row r="23" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D23" s="3"/>
-      <c r="AQ23" s="1"/>
+    <row r="23" spans="4:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D23" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
+      <c r="L23" s="6"/>
+      <c r="M23" s="6"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="6"/>
+      <c r="P23" s="6"/>
+      <c r="Q23" s="6"/>
+      <c r="R23" s="6"/>
+      <c r="S23" s="6"/>
+      <c r="T23" s="6"/>
+      <c r="U23" s="6"/>
+      <c r="V23" s="6"/>
+      <c r="W23" s="6"/>
+      <c r="X23" s="6"/>
+      <c r="Y23" s="6"/>
+      <c r="Z23" s="6"/>
+      <c r="AA23" s="6"/>
+      <c r="AB23" s="6"/>
+      <c r="AC23" s="6"/>
+      <c r="AD23" s="6"/>
+      <c r="AE23" s="6"/>
+      <c r="AF23" s="6"/>
+      <c r="AG23" s="6"/>
+      <c r="AH23" s="6"/>
+      <c r="AI23" s="6"/>
+      <c r="AJ23" s="6"/>
+      <c r="AK23" s="6"/>
+      <c r="AL23" s="6"/>
+      <c r="AM23" s="6"/>
+      <c r="AN23" s="6"/>
+      <c r="AO23" s="6"/>
+      <c r="AP23" s="6"/>
+      <c r="AQ23" s="7"/>
     </row>
     <row r="24" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D24" s="3"/>
@@ -1120,56 +1814,18 @@
       <c r="D25" s="3"/>
       <c r="AQ25" s="1"/>
     </row>
-    <row r="26" spans="4:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D26" s="3"/>
       <c r="AQ26" s="1"/>
     </row>
-    <row r="27" spans="4:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D27" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
-      <c r="L27" s="5"/>
-      <c r="M27" s="5"/>
-      <c r="N27" s="5"/>
-      <c r="O27" s="5"/>
-      <c r="P27" s="5"/>
-      <c r="Q27" s="5"/>
-      <c r="R27" s="5"/>
-      <c r="S27" s="5"/>
-      <c r="T27" s="5"/>
-      <c r="U27" s="5"/>
-      <c r="V27" s="5"/>
-      <c r="W27" s="5"/>
-      <c r="X27" s="5"/>
-      <c r="Y27" s="5"/>
-      <c r="Z27" s="5"/>
-      <c r="AA27" s="5"/>
-      <c r="AB27" s="5"/>
-      <c r="AC27" s="5"/>
-      <c r="AD27" s="5"/>
-      <c r="AE27" s="5"/>
-      <c r="AF27" s="5"/>
-      <c r="AG27" s="5"/>
-      <c r="AH27" s="5"/>
-      <c r="AI27" s="5"/>
-      <c r="AJ27" s="5"/>
-      <c r="AK27" s="5"/>
-      <c r="AL27" s="5"/>
-      <c r="AM27" s="5"/>
-      <c r="AN27" s="5"/>
-      <c r="AO27" s="5"/>
-      <c r="AP27" s="5"/>
-      <c r="AQ27" s="6"/>
-    </row>
     <row r="28" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D28" s="3"/>
+      <c r="G28" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="Z28" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="AQ28" s="1"/>
     </row>
     <row r="29" spans="4:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -1246,99 +1902,9 @@
       <c r="D46" s="3"/>
       <c r="AQ46" s="1"/>
     </row>
-    <row r="47" spans="4:52" ht="26.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="4:52" ht="36.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="49" spans="4:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D49" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5"/>
-      <c r="G49" s="5"/>
-      <c r="H49" s="5"/>
-      <c r="I49" s="5"/>
-      <c r="J49" s="5"/>
-      <c r="K49" s="5"/>
-      <c r="L49" s="5"/>
-      <c r="M49" s="5"/>
-      <c r="N49" s="5"/>
-      <c r="O49" s="5"/>
-      <c r="P49" s="5"/>
-      <c r="Q49" s="5"/>
-      <c r="R49" s="5"/>
-      <c r="S49" s="5"/>
-      <c r="T49" s="5"/>
-      <c r="U49" s="5"/>
-      <c r="V49" s="5"/>
-      <c r="W49" s="5"/>
-      <c r="X49" s="5"/>
-      <c r="Y49" s="5"/>
-      <c r="Z49" s="5"/>
-      <c r="AA49" s="5"/>
-      <c r="AB49" s="5"/>
-      <c r="AC49" s="5"/>
-      <c r="AD49" s="5"/>
-      <c r="AE49" s="5"/>
-      <c r="AF49" s="5"/>
-      <c r="AG49" s="5"/>
-      <c r="AH49" s="5"/>
-      <c r="AI49" s="5"/>
-      <c r="AJ49" s="5"/>
-      <c r="AK49" s="5"/>
-      <c r="AL49" s="5"/>
-      <c r="AM49" s="5"/>
-      <c r="AN49" s="5"/>
-      <c r="AO49" s="5"/>
-      <c r="AP49" s="5"/>
-      <c r="AQ49" s="6"/>
-    </row>
-    <row r="69" spans="4:52" ht="23.25" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="4:52" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="71" spans="4:52" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D71" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E71" s="5"/>
-      <c r="F71" s="5"/>
-      <c r="G71" s="5"/>
-      <c r="H71" s="5"/>
-      <c r="I71" s="5"/>
-      <c r="J71" s="5"/>
-      <c r="K71" s="5"/>
-      <c r="L71" s="5"/>
-      <c r="M71" s="5"/>
-      <c r="N71" s="5"/>
-      <c r="O71" s="5"/>
-      <c r="P71" s="5"/>
-      <c r="Q71" s="5"/>
-      <c r="R71" s="5"/>
-      <c r="S71" s="5"/>
-      <c r="T71" s="5"/>
-      <c r="U71" s="5"/>
-      <c r="V71" s="5"/>
-      <c r="W71" s="5"/>
-      <c r="X71" s="5"/>
-      <c r="Y71" s="5"/>
-      <c r="Z71" s="5"/>
-      <c r="AA71" s="5"/>
-      <c r="AB71" s="5"/>
-      <c r="AC71" s="5"/>
-      <c r="AD71" s="5"/>
-      <c r="AE71" s="5"/>
-      <c r="AF71" s="5"/>
-      <c r="AG71" s="5"/>
-      <c r="AH71" s="5"/>
-      <c r="AI71" s="5"/>
-      <c r="AJ71" s="5"/>
-      <c r="AK71" s="5"/>
-      <c r="AL71" s="5"/>
-      <c r="AM71" s="5"/>
-      <c r="AN71" s="5"/>
-      <c r="AO71" s="5"/>
-      <c r="AP71" s="5"/>
-      <c r="AQ71" s="6"/>
-    </row>
-    <row r="77" spans="4:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="4:52" ht="36.6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="52:52" ht="23.25" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="52:52" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="AZ77"/>
     </row>
     <row r="91" spans="53:53" ht="23.25" x14ac:dyDescent="0.25"/>
@@ -1354,21 +1920,9 @@
     <row r="136" ht="23.25" x14ac:dyDescent="0.25"/>
     <row r="157" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="D49:AQ49"/>
-    <mergeCell ref="D71:AQ71"/>
-    <mergeCell ref="D6:AQ6"/>
-    <mergeCell ref="D27:AQ27"/>
+  <mergeCells count="2">
+    <mergeCell ref="D23:AQ23"/>
     <mergeCell ref="D1:AQ1"/>
-    <mergeCell ref="K3:O3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="AD3:AK3"/>
-    <mergeCell ref="D5:AQ5"/>
-    <mergeCell ref="D4:AQ4"/>
-    <mergeCell ref="D3:J3"/>
-    <mergeCell ref="D2:AQ2"/>
-    <mergeCell ref="AL3:AQ3"/>
-    <mergeCell ref="X3:AC3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>
@@ -1376,14 +1930,25 @@
   <headerFooter scaleWithDoc="0" alignWithMargins="0">
     <oddFooter>&amp;L&amp;"Arial,Bold"&amp;12Appendix B &amp;"Arial,Regular"- Page &amp;"Arial,Bold"&amp;P &amp;"Arial,Regular"of&amp;"Arial,Bold" &amp;N&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;22&amp;K0073CF INTERNAL</oddFooter>
   </headerFooter>
-  <rowBreaks count="1" manualBreakCount="1">
-    <brk id="48" min="3" max="42" man="1"/>
-  </rowBreaks>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BA3B7D55240AD64FBD207B9711FF53CE" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6be4015347e02ecebfa52d44e62f8e86">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="2feb5366-15dc-478f-8d1e-b18e91183cdf" xmlns:ns4="aad71146-b4dd-4159-beac-3e7532a143d7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="241b9938227cbf8a4c3099596e0f279f" ns3:_="" ns4:_="">
     <xsd:import namespace="2feb5366-15dc-478f-8d1e-b18e91183cdf"/>
@@ -1606,22 +2171,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8595652-F5B8-490F-926E-A88B88209135}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2feb5366-15dc-478f-8d1e-b18e91183cdf"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="aad71146-b4dd-4159-beac-3e7532a143d7"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{563C90C2-C70F-4E90-9E41-58DA15D92D43}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3B565BB7-800B-452C-9D98-5C0B0C0C8F10}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1638,29 +2213,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{563C90C2-C70F-4E90-9E41-58DA15D92D43}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8595652-F5B8-490F-926E-A88B88209135}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="2feb5366-15dc-478f-8d1e-b18e91183cdf"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="aad71146-b4dd-4159-beac-3e7532a143d7"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>